<commit_message>
Actualizacion asignaciones - 2026-07-15 15:56:43
</commit_message>
<xml_diff>
--- a/MANTENIMIENTO/Formato de mantenimiento preventivo.xlsx
+++ b/MANTENIMIENTO/Formato de mantenimiento preventivo.xlsx
@@ -50980,11 +50980,7 @@
       <c r="A2" t="n">
         <v>392368</v>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>NESTOR LEONARDO CORTES TORRES</t>
-        </is>
-      </c>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
           <t>Pendiente</t>
@@ -51205,7 +51201,11 @@
       <c r="A15" t="n">
         <v>392368</v>
       </c>
-      <c r="B15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>NESTOR LEONARDO CORTES TORRES</t>
+        </is>
+      </c>
       <c r="C15" t="inlineStr">
         <is>
           <t>Pendiente</t>

</xml_diff>

<commit_message>
Actualizacion asignaciones - 2026-07-15 16:00:18
</commit_message>
<xml_diff>
--- a/MANTENIMIENTO/Formato de mantenimiento preventivo.xlsx
+++ b/MANTENIMIENTO/Formato de mantenimiento preventivo.xlsx
@@ -51201,11 +51201,7 @@
       <c r="A15" t="n">
         <v>392368</v>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>NESTOR LEONARDO CORTES TORRES</t>
-        </is>
-      </c>
+      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>Pendiente</t>

</xml_diff>

<commit_message>
Actualizacion asignaciones - 2026-07-15 16:00:23
</commit_message>
<xml_diff>
--- a/MANTENIMIENTO/Formato de mantenimiento preventivo.xlsx
+++ b/MANTENIMIENTO/Formato de mantenimiento preventivo.xlsx
@@ -50980,7 +50980,11 @@
       <c r="A2" t="n">
         <v>392368</v>
       </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>NESTOR LEONARDO CORTES TORRES</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>Pendiente</t>

</xml_diff>

<commit_message>
Actualizacion asignaciones - 2026-07-15 16:01:05
</commit_message>
<xml_diff>
--- a/MANTENIMIENTO/Formato de mantenimiento preventivo.xlsx
+++ b/MANTENIMIENTO/Formato de mantenimiento preventivo.xlsx
@@ -50980,11 +50980,7 @@
       <c r="A2" t="n">
         <v>392368</v>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>NESTOR LEONARDO CORTES TORRES</t>
-        </is>
-      </c>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
           <t>Pendiente</t>
@@ -51205,7 +51201,11 @@
       <c r="A15" t="n">
         <v>392368</v>
       </c>
-      <c r="B15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>NESTOR LEONARDO CORTES TORRES</t>
+        </is>
+      </c>
       <c r="C15" t="inlineStr">
         <is>
           <t>Pendiente</t>

</xml_diff>

<commit_message>
Actualizacion asignaciones - 2026-07-15 16:02:43
</commit_message>
<xml_diff>
--- a/MANTENIMIENTO/Formato de mantenimiento preventivo.xlsx
+++ b/MANTENIMIENTO/Formato de mantenimiento preventivo.xlsx
@@ -51211,12 +51211,28 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Rojo</t>
+        </is>
+      </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">

</xml_diff>

<commit_message>
Actualizacion asignaciones - 2026-07-15 16:03:58
</commit_message>
<xml_diff>
--- a/MANTENIMIENTO/Formato de mantenimiento preventivo.xlsx
+++ b/MANTENIMIENTO/Formato de mantenimiento preventivo.xlsx
@@ -50980,7 +50980,11 @@
       <c r="A2" t="n">
         <v>392368</v>
       </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>NESTOR LEONARDO CORTES TORRES</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>Pendiente</t>
@@ -51201,38 +51205,18 @@
       <c r="A15" t="n">
         <v>392368</v>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>NESTOR LEONARDO CORTES TORRES</t>
-        </is>
-      </c>
+      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Rojo</t>
-        </is>
-      </c>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>08:00</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">

</xml_diff>

<commit_message>
Actualizacion asignaciones - 2026-07-15 16:04:41
</commit_message>
<xml_diff>
--- a/MANTENIMIENTO/Formato de mantenimiento preventivo.xlsx
+++ b/MANTENIMIENTO/Formato de mantenimiento preventivo.xlsx
@@ -50980,11 +50980,7 @@
       <c r="A2" t="n">
         <v>392368</v>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>NESTOR LEONARDO CORTES TORRES</t>
-        </is>
-      </c>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
           <t>Pendiente</t>
@@ -51205,7 +51201,11 @@
       <c r="A15" t="n">
         <v>392368</v>
       </c>
-      <c r="B15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>NESTOR LEONARDO CORTES TORRES</t>
+        </is>
+      </c>
       <c r="C15" t="inlineStr">
         <is>
           <t>Pendiente</t>

</xml_diff>